<commit_message>
Remove the CBC variant of the MILP method
- Keep one MILP solver (HiGHS). CBC used the same model and gave worse results.
- Remove the milp_cbc rows and solutions from the results.
- Rebuild the comparison figures and the demo notebook.
</commit_message>
<xml_diff>
--- a/results/schedule_M_s1.xlsx
+++ b/results/schedule_M_s1.xlsx
@@ -951,16 +951,16 @@
         <v>28</v>
       </c>
       <c r="G15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K15" t="inlineStr"/>
     </row>
@@ -992,10 +992,10 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J16" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="K16" t="inlineStr"/>
     </row>
@@ -1027,10 +1027,10 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J17" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K17" t="inlineStr"/>
     </row>
@@ -1056,10 +1056,10 @@
         <v>28</v>
       </c>
       <c r="G18" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>116</v>
@@ -1196,16 +1196,16 @@
         <v>32</v>
       </c>
       <c r="G22" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H22" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J22" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K22" t="inlineStr"/>
     </row>
@@ -1237,10 +1237,10 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J23" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K23" t="inlineStr"/>
     </row>
@@ -1266,10 +1266,10 @@
         <v>32</v>
       </c>
       <c r="G24" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I24" t="n">
         <v>105</v>
@@ -1371,16 +1371,16 @@
         <v>5</v>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I27" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J27" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K27" t="inlineStr"/>
     </row>
@@ -1406,10 +1406,10 @@
         <v>30</v>
       </c>
       <c r="G28" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
         <v>33</v>
@@ -1756,16 +1756,16 @@
         <v>30</v>
       </c>
       <c r="G38" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I38" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J38" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K38" t="inlineStr"/>
     </row>
@@ -1797,10 +1797,10 @@
         <v>0</v>
       </c>
       <c r="I39" t="n">
+        <v>142</v>
+      </c>
+      <c r="J39" t="n">
         <v>143</v>
-      </c>
-      <c r="J39" t="n">
-        <v>144</v>
       </c>
       <c r="K39" t="inlineStr"/>
     </row>
@@ -1832,10 +1832,10 @@
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J40" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K40" t="inlineStr"/>
     </row>
@@ -2001,16 +2001,16 @@
         <v>38</v>
       </c>
       <c r="G45" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J45" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K45" t="inlineStr"/>
     </row>
@@ -2106,16 +2106,16 @@
         <v>34</v>
       </c>
       <c r="G48" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I48" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J48" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="K48" t="inlineStr"/>
     </row>
@@ -2147,10 +2147,10 @@
         <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="J49" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="K49" t="inlineStr"/>
     </row>
@@ -2176,10 +2176,10 @@
         <v>34</v>
       </c>
       <c r="G50" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H50" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
         <v>127</v>
@@ -2246,16 +2246,16 @@
         <v>33</v>
       </c>
       <c r="G52" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H52" t="n">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="I52" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J52" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="K52" t="inlineStr"/>
     </row>
@@ -2281,16 +2281,16 @@
         <v>38</v>
       </c>
       <c r="G53" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I53" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="J53" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="K53" t="inlineStr"/>
     </row>
@@ -2322,10 +2322,10 @@
         <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="J54" t="n">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="K54" t="inlineStr"/>
     </row>
@@ -2357,10 +2357,10 @@
         <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="J55" t="n">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="K55" t="inlineStr"/>
     </row>
@@ -2392,10 +2392,10 @@
         <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="J56" t="n">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="K56" t="inlineStr"/>
     </row>

</xml_diff>